<commit_message>
tried updating roi centers; not stable
</commit_message>
<xml_diff>
--- a/data_overview.xlsx
+++ b/data_overview.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\jkerssemakers\Dropbox\CD_recent\BN_CD23_Rafael\analysis\CD23_Rafa\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F02FF4E7-0BC1-4260-AAC2-3E14D2AE94EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68CBE833-CFCD-47F8-90FC-90FB48056FD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3810" yWindow="1185" windowWidth="9315" windowHeight="12945" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="495" yWindow="1005" windowWidth="9315" windowHeight="12945" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="general" sheetId="1" r:id="rId1"/>
@@ -761,7 +761,7 @@
         <v>20</v>
       </c>
       <c r="D8" s="2">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="E8">
         <v>0</v>

</xml_diff>

<commit_message>
refining processed data; add time calib
</commit_message>
<xml_diff>
--- a/data_overview.xlsx
+++ b/data_overview.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\jkerssemakers\Dropbox\CD_recent\BN_CD23_Rafael\analysis\CD23_Rafa\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1138A0F-F072-41C5-A767-4FF662094B68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24EA889D-DAEC-4717-8157-A68EB77279B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="240" windowWidth="9315" windowHeight="12945" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="general" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
   <si>
     <t>run index</t>
   </si>
@@ -203,6 +203,9 @@
   </si>
   <si>
     <t>movie_id</t>
+  </si>
+  <si>
+    <t>dt(s)</t>
   </si>
 </sst>
 </file>
@@ -236,12 +239,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -256,7 +265,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -265,6 +274,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -622,7 +632,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{033352EE-E1CE-4541-B0CC-785AB457CDEA}">
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.42578125" customWidth="1"/>
@@ -632,7 +642,7 @@
     <col min="5" max="5" width="12.42578125" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>57</v>
       </c>
@@ -648,12 +658,15 @@
       <c r="E1" s="3" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>5</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="4">
         <v>462</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -665,12 +678,15 @@
       <c r="E2" s="3">
         <v>1000000</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>5</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="4">
         <v>462</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -682,12 +698,15 @@
       <c r="E3" s="3">
         <v>33</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>5</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="4">
         <v>462</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -699,12 +718,15 @@
       <c r="E4" s="3">
         <v>30</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>5</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="4">
         <v>462</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -716,12 +738,15 @@
       <c r="E5" s="3">
         <v>30</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="4">
         <v>462</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -733,12 +758,15 @@
       <c r="E6" s="3">
         <v>1000000</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="4">
         <v>462</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -750,12 +778,15 @@
       <c r="E7" s="3">
         <v>30</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>5</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="4">
         <v>462</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -767,12 +798,15 @@
       <c r="E8" s="3">
         <v>1000000</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>5</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="4">
         <v>462</v>
       </c>
       <c r="C9" s="2" t="s">
@@ -784,12 +818,15 @@
       <c r="E9" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>5</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="4">
         <v>462</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -801,12 +838,15 @@
       <c r="E10" s="3">
         <v>40</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F10">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>5</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="4">
         <v>462</v>
       </c>
       <c r="C11" s="2" t="s">
@@ -818,12 +858,15 @@
       <c r="E11" s="3">
         <v>21</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>5</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="4">
         <v>462</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -835,12 +878,15 @@
       <c r="E12" s="3">
         <v>1000000</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F12">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>5</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="4">
         <v>462</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -852,12 +898,15 @@
       <c r="E13" s="3">
         <v>1000000</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F13">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>5</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="4">
         <v>462</v>
       </c>
       <c r="C14" s="2" t="s">
@@ -869,12 +918,15 @@
       <c r="E14" s="3">
         <v>1000000</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F14">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>5</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="4">
         <v>462</v>
       </c>
       <c r="C15" s="2" t="s">
@@ -886,12 +938,15 @@
       <c r="E15" s="3">
         <v>55</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F15">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>5</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="4">
         <v>462</v>
       </c>
       <c r="C16" s="2" t="s">
@@ -903,12 +958,15 @@
       <c r="E16" s="3">
         <v>40</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F16">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>5</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="4">
         <v>462</v>
       </c>
       <c r="C17" s="2" t="s">
@@ -920,12 +978,15 @@
       <c r="E17" s="3">
         <v>1000000</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F17">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>5</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="4">
         <v>462</v>
       </c>
       <c r="C18" s="2" t="s">
@@ -937,8 +998,11 @@
       <c r="E18" s="3">
         <v>1000000</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F18">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>5</v>
       </c>
@@ -954,8 +1018,11 @@
       <c r="E19" s="3">
         <v>1000000</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>5</v>
       </c>
@@ -971,8 +1038,11 @@
       <c r="E20" s="3">
         <v>14</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>5</v>
       </c>
@@ -988,8 +1058,11 @@
       <c r="E21" s="3">
         <v>100</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F21">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>5</v>
       </c>
@@ -1005,8 +1078,11 @@
       <c r="E22" s="3">
         <v>1000000</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>5</v>
       </c>
@@ -1022,8 +1098,11 @@
       <c r="E23" s="3">
         <v>79</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F23">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>5</v>
       </c>
@@ -1039,8 +1118,11 @@
       <c r="E24" s="3">
         <v>79</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F24">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>5</v>
       </c>
@@ -1056,8 +1138,11 @@
       <c r="E25" s="3">
         <v>79</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>5</v>
       </c>
@@ -1073,8 +1158,11 @@
       <c r="E26" s="3">
         <v>75</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F26">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>5</v>
       </c>
@@ -1090,8 +1178,11 @@
       <c r="E27" s="3">
         <v>1000000</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F27">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>5</v>
       </c>
@@ -1107,12 +1198,15 @@
       <c r="E28" s="3">
         <v>175</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F28">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>5</v>
       </c>
-      <c r="B29">
+      <c r="B29" s="4">
         <v>465</v>
       </c>
       <c r="C29" s="2" t="s">
@@ -1124,12 +1218,15 @@
       <c r="E29" s="3">
         <v>20</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>5</v>
       </c>
-      <c r="B30">
+      <c r="B30" s="4">
         <v>465</v>
       </c>
       <c r="C30" s="2" t="s">
@@ -1141,12 +1238,15 @@
       <c r="E30" s="3">
         <v>50</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F30">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>5</v>
       </c>
-      <c r="B31">
+      <c r="B31" s="4">
         <v>465</v>
       </c>
       <c r="C31" s="2" t="s">
@@ -1158,12 +1258,15 @@
       <c r="E31" s="3">
         <v>1000000</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F31">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>5</v>
       </c>
-      <c r="B32">
+      <c r="B32" s="4">
         <v>465</v>
       </c>
       <c r="C32" s="2" t="s">
@@ -1175,12 +1278,15 @@
       <c r="E32" s="3">
         <v>1000000</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F32">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>5</v>
       </c>
-      <c r="B33">
+      <c r="B33" s="4">
         <v>465</v>
       </c>
       <c r="C33" s="2" t="s">
@@ -1192,12 +1298,15 @@
       <c r="E33" s="3">
         <v>1000000</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F33">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>5</v>
       </c>
-      <c r="B34">
+      <c r="B34" s="4">
         <v>465</v>
       </c>
       <c r="C34" s="2" t="s">
@@ -1209,12 +1318,15 @@
       <c r="E34" s="3">
         <v>20</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F34">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>5</v>
       </c>
-      <c r="B35">
+      <c r="B35" s="4">
         <v>465</v>
       </c>
       <c r="C35" s="2" t="s">
@@ -1226,8 +1338,11 @@
       <c r="E35" s="3">
         <v>1000000</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F35">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>5</v>
       </c>
@@ -1243,8 +1358,11 @@
       <c r="E36" s="3">
         <v>50</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F36">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>5</v>
       </c>
@@ -1260,8 +1378,11 @@
       <c r="E37" s="3">
         <v>80</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F37">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>5</v>
       </c>
@@ -1277,8 +1398,11 @@
       <c r="E38" s="3">
         <v>1000000</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F38">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>5</v>
       </c>
@@ -1294,8 +1418,11 @@
       <c r="E39" s="3">
         <v>1000000</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F39">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>5</v>
       </c>
@@ -1311,8 +1438,11 @@
       <c r="E40" s="3">
         <v>1000000</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F40">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>5</v>
       </c>
@@ -1328,8 +1458,11 @@
       <c r="E41" s="3">
         <v>1000000</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F41">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>5</v>
       </c>
@@ -1344,6 +1477,9 @@
       </c>
       <c r="E42" s="3">
         <v>1000000</v>
+      </c>
+      <c r="F42">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>